<commit_message>
Add five graded structured questions per topic
Each topic now has five structured questions, from Level 1 (easy) to
Level 5 (challenge), with full worked answers in the answer key.
Existing questions were renumbered into the new sequence, and the
Excel practice sheets now point to the new question numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cg2FRYV2NgKh9WWDoLcpR2
</commit_message>
<xml_diff>
--- a/excel/Ch08_Irrecoverable_Debts.xlsx
+++ b/excel/Ch08_Irrecoverable_Debts.xlsx
@@ -176,7 +176,7 @@
     <t xml:space="preserve">Year ended 31 December 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice: Model Question 8.8 (Grace)</t>
+    <t xml:space="preserve">Practice: Model Question 8.11 (Grace)</t>
   </si>
   <si>
     <t xml:space="preserve">Type your answers in the yellow cells. The Check column marks them.</t>
@@ -185,7 +185,7 @@
     <t xml:space="preserve">Grace keeps an allowance for irrecoverable debts. Year end 31 December.</t>
   </si>
   <si>
-    <t xml:space="preserve">Data (from Model Question 8.8)</t>
+    <t xml:space="preserve">Data (from Model Question 8.11)</t>
   </si>
   <si>
     <t xml:space="preserve">Debts to be written off</t>
@@ -248,7 +248,7 @@
     <t xml:space="preserve">Your score (number correct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice: Model Question 8.8 (Grace): Answers</t>
+    <t xml:space="preserve">Practice: Model Question 8.11 (Grace): Answers</t>
   </si>
   <si>
     <t xml:space="preserve">Every answer is a formula linked to the Practice sheet data.</t>

</xml_diff>